<commit_message>
UCONN walkways: base estimate on drawings only - no photographs were provided
The client's email offered photos but none were sent. Removed photograph
reliance from the letter (scope, documents and quantities assumptions), the
analysis record, and the estimate line rationale; repriced (fee unchanged at
$9,050 incl. optional site visit, new lock 77b64f13667b) and refreshed the
buildup workbook and proposal database record.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mP1iTukX1sv7YH1yyeg1v
</commit_message>
<xml_diff>
--- a/jobs/uconn-walkways/out/fee_buildup.xlsx
+++ b/jobs/uconn-walkways/out/fee_buildup.xlsx
@@ -74,7 +74,7 @@
     <t xml:space="preserve">CD-Level Cost Estimate — Connector Walkway &amp; Chimney Repairs  [A]</t>
   </si>
   <si>
-    <t xml:space="preserve">Kickoff; review 6-sheet CD Review set and photographs; clarification/RFI list to architect</t>
+    <t xml:space="preserve">Kickoff; review 6-sheet CD Review set; clarification/RFI list to architect</t>
   </si>
   <si>
     <t xml:space="preserve">A</t>
@@ -137,7 +137,7 @@
     <t xml:space="preserve">TOTAL LUMP SUM FEE</t>
   </si>
   <si>
-    <t xml:space="preserve">Locked fee model a9a64e82bcc4: total $9,050. If the buildup is edited, re-run `feeprop price` so the proposal and this workbook stay on one number.</t>
+    <t xml:space="preserve">Locked fee model 77b64f13667b: total $9,050. If the buildup is edited, re-run `feeprop price` so the proposal and this workbook stay on one number.</t>
   </si>
 </sst>
 </file>
@@ -544,7 +544,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="3" t="s">
         <v>17</v>
       </c>

</xml_diff>